<commit_message>
update with more options for geolocalization
</commit_message>
<xml_diff>
--- a/examples/berlin_out/enriched_addresses.xlsx
+++ b/examples/berlin_out/enriched_addresses.xlsx
@@ -494,10 +494,10 @@
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="n">
-        <v>52.5314585</v>
+        <v>52.5286468</v>
       </c>
       <c r="I2" t="n">
-        <v>13.386998</v>
+        <v>13.3766197</v>
       </c>
     </row>
     <row r="3">
@@ -531,10 +531,10 @@
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="n">
-        <v>52.533095</v>
+        <v>52.5345286</v>
       </c>
       <c r="I3" t="n">
-        <v>13.4144592</v>
+        <v>13.41605</v>
       </c>
     </row>
     <row r="4">

</xml_diff>